<commit_message>
Updated: Merge CSV Funds results
</commit_message>
<xml_diff>
--- a/spreadsheet/charles_stanley.xlsx
+++ b/spreadsheet/charles_stanley.xlsx
@@ -435,21 +435,31 @@
           <t>https://www.charles-stanley-direct.co.uk/ViewFund?InvestmentId=G9%2BpUE7%2BaEg%3D&amp;Isin=GB00B2PB2C75&amp;PreviousSearchResults=%2FInvestmentSearch%2FSearch%3FSearchType%3DKeywordSearch%26Category%3DFunds%26SortColumn%3DName%26SortDirection%3DAsc%26Pagesize%3D50%26Page%3D1</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Invest in this fund within an ISA, JISA, SIPP or Investment Account</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="18" customFormat="1" customHeight="1" s="6">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>7IM AAP Adventurous C Inc</t>
+          <t>7IM Adventurous C Acc</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>GB00B2PB2B68</t>
+          <t>GB0033958009</t>
         </is>
       </c>
       <c r="C3" s="9" t="inlineStr">
         <is>
-          <t>https://www.charles-stanley-direct.co.uk/ViewFund?InvestmentId=YU2xRK6U3r0%3D&amp;Isin=GB00B2PB2B68&amp;PreviousSearchResults=%2FInvestmentSearch%2FSearch%3FSearchType%3DKeywordSearch%26Category%3DFunds%26SortColumn%3DName%26SortDirection%3DAsc%26Pagesize%3D50%26Page%3D1</t>
+          <t>https://www.charles-stanley-direct.co.uk/ViewFund?InvestmentId=geMXjfW4gYY%3D&amp;Isin=GB0033958009&amp;PreviousSearchResults=%2FInvestmentSearch%2FSearch%3FSearchType%3DKeywordSearch%26Category%3DFunds%26SortColumn%3DName%26SortDirection%3DAsc%26Pagesize%3D50%26Page%3D1</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Invest in this fund within an ISA, JISA, SIPP or Investment Account</t>
         </is>
       </c>
     </row>

</xml_diff>